<commit_message>
fix(excel): preserve detail sheet layout and prevent breaker isolation column deformation
</commit_message>
<xml_diff>
--- a/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
+++ b/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
@@ -9778,7 +9778,8 @@
     <mergeCell ref="O17:S17"/>
     <mergeCell ref="O11:S11"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -10779,8 +10780,8 @@
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="J40:Q40"/>
     <mergeCell ref="B5:Q5"/>
-    <mergeCell ref="J40:Q40"/>
     <mergeCell ref="H16:J16"/>
     <mergeCell ref="D37:Q38"/>
     <mergeCell ref="K3:Q3"/>
@@ -10823,7 +10824,8 @@
     <mergeCell ref="K2:Q2"/>
     <mergeCell ref="K18:L18"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -12147,8 +12149,8 @@
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="F25:I25"/>
+    <mergeCell ref="N39:O39"/>
     <mergeCell ref="B8:I8"/>
-    <mergeCell ref="N39:O39"/>
     <mergeCell ref="J19:M19"/>
     <mergeCell ref="P39:Q39"/>
     <mergeCell ref="J28:M28"/>
@@ -12264,7 +12266,8 @@
     <mergeCell ref="K2:Q2"/>
     <mergeCell ref="N36:O36"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -13795,8 +13798,8 @@
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="J9:L9"/>
     <mergeCell ref="B28:E28"/>
+    <mergeCell ref="I27:I28"/>
     <mergeCell ref="W38:AJ38"/>
-    <mergeCell ref="I27:I28"/>
     <mergeCell ref="J23:Q23"/>
     <mergeCell ref="W28:AD28"/>
     <mergeCell ref="N19:Q19"/>
@@ -13817,7 +13820,8 @@
     <mergeCell ref="W42:AJ42"/>
     <mergeCell ref="K2:Q2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -15313,7 +15317,8 @@
     <mergeCell ref="O30:Q30"/>
     <mergeCell ref="B13:Q13"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -16561,7 +16566,8 @@
     <mergeCell ref="L36:M36"/>
     <mergeCell ref="E21:F21"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -27560,7 +27566,8 @@
     <mergeCell ref="H25:J25"/>
     <mergeCell ref="H26:I26"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -29115,8 +29122,8 @@
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="N22:O22"/>
+    <mergeCell ref="P22:Q22"/>
     <mergeCell ref="J11:L11"/>
-    <mergeCell ref="P22:Q22"/>
     <mergeCell ref="V20:W20"/>
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="K17:M17"/>
@@ -29134,8 +29141,8 @@
     <mergeCell ref="J2:Q2"/>
     <mergeCell ref="H23:I23"/>
     <mergeCell ref="J23:K23"/>
+    <mergeCell ref="D26:E26"/>
     <mergeCell ref="B16:B19"/>
-    <mergeCell ref="D26:E26"/>
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="P26:Q26"/>
     <mergeCell ref="V3:AC3"/>
@@ -29242,7 +29249,8 @@
     <mergeCell ref="V18:W18"/>
     <mergeCell ref="H26:I26"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -30942,8 +30950,8 @@
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="N22:O22"/>
+    <mergeCell ref="P22:Q22"/>
     <mergeCell ref="J11:L11"/>
-    <mergeCell ref="P22:Q22"/>
     <mergeCell ref="V20:W20"/>
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="K17:M17"/>
@@ -30961,8 +30969,8 @@
     <mergeCell ref="J2:Q2"/>
     <mergeCell ref="H23:I23"/>
     <mergeCell ref="J23:K23"/>
+    <mergeCell ref="D26:E26"/>
     <mergeCell ref="B16:B19"/>
-    <mergeCell ref="D26:E26"/>
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="P26:Q26"/>
     <mergeCell ref="V3:AC3"/>
@@ -31069,7 +31077,8 @@
     <mergeCell ref="V18:W18"/>
     <mergeCell ref="H26:I26"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.3543307086614173" bottom="0.3543307086614173" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(breaker): complete breaker form fields, dates and original layout
</commit_message>
<xml_diff>
--- a/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
+++ b/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
@@ -10780,8 +10780,8 @@
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B5:Q5"/>
     <mergeCell ref="J40:Q40"/>
-    <mergeCell ref="B5:Q5"/>
     <mergeCell ref="H16:J16"/>
     <mergeCell ref="D37:Q38"/>
     <mergeCell ref="K3:Q3"/>
@@ -12149,8 +12149,8 @@
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="F25:I25"/>
+    <mergeCell ref="B8:I8"/>
     <mergeCell ref="N39:O39"/>
-    <mergeCell ref="B8:I8"/>
     <mergeCell ref="J19:M19"/>
     <mergeCell ref="P39:Q39"/>
     <mergeCell ref="J28:M28"/>
@@ -13798,8 +13798,8 @@
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="J9:L9"/>
     <mergeCell ref="B28:E28"/>
+    <mergeCell ref="W38:AJ38"/>
     <mergeCell ref="I27:I28"/>
-    <mergeCell ref="W38:AJ38"/>
     <mergeCell ref="J23:Q23"/>
     <mergeCell ref="W28:AD28"/>
     <mergeCell ref="N19:Q19"/>
@@ -29122,8 +29122,8 @@
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="N22:O22"/>
+    <mergeCell ref="J11:L11"/>
     <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="J11:L11"/>
     <mergeCell ref="V20:W20"/>
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="K17:M17"/>
@@ -29141,8 +29141,8 @@
     <mergeCell ref="J2:Q2"/>
     <mergeCell ref="H23:I23"/>
     <mergeCell ref="J23:K23"/>
+    <mergeCell ref="B16:B19"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B16:B19"/>
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="P26:Q26"/>
     <mergeCell ref="V3:AC3"/>
@@ -30950,8 +30950,8 @@
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="N22:O22"/>
+    <mergeCell ref="J11:L11"/>
     <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="J11:L11"/>
     <mergeCell ref="V20:W20"/>
     <mergeCell ref="H19:J19"/>
     <mergeCell ref="K17:M17"/>
@@ -30969,8 +30969,8 @@
     <mergeCell ref="J2:Q2"/>
     <mergeCell ref="H23:I23"/>
     <mergeCell ref="J23:K23"/>
+    <mergeCell ref="B16:B19"/>
     <mergeCell ref="D26:E26"/>
-    <mergeCell ref="B16:B19"/>
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="P26:Q26"/>
     <mergeCell ref="V3:AC3"/>

</xml_diff>

<commit_message>
fix(templates): update grounding resistance limit criteria to 4 Ohm in TOPRAKLAMALAR sheet
</commit_message>
<xml_diff>
--- a/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
+++ b/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
@@ -2910,7 +2910,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3063,7 +3063,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -3108,7 +3108,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3348,7 +3348,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3501,7 +3501,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -3546,7 +3546,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3626,7 +3626,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3695,7 +3695,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3787,7 +3787,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3905,7 +3905,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3988,7 +3988,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4057,7 +4057,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4149,7 +4149,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4267,7 +4267,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4357,7 +4357,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4430,7 +4430,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4522,7 +4522,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4640,7 +4640,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4723,7 +4723,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4820,7 +4820,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4932,7 +4932,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -4994,7 +4994,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -5033,7 +5033,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -6664,25 +6664,11 @@
     <row r="30" s="227"/>
     <row r="31"/>
     <row r="32" ht="11.25" customHeight="1" s="227"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40" s="227"/>
     <row r="41" s="227"/>
     <row r="42" s="227"/>
-    <row r="43"/>
     <row r="44" s="227"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
     <row r="48" ht="7.5" customHeight="1" s="227"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="481" t="n"/>
       <c r="B52" s="99" t="n"/>
@@ -26490,7 +26476,7 @@
       </c>
       <c r="C16" s="482" t="n"/>
       <c r="D16" s="515" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="482" t="n"/>
       <c r="F16" s="516" t="inlineStr">
@@ -26747,7 +26733,7 @@
       </c>
       <c r="E26" s="99" t="n"/>
       <c r="F26" s="525" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G26" s="526" t="inlineStr">
         <is>
@@ -26804,7 +26790,7 @@
       </c>
       <c r="E27" s="99" t="n"/>
       <c r="F27" s="525" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G27" s="526" t="inlineStr">
         <is>
@@ -26861,7 +26847,7 @@
       </c>
       <c r="E28" s="99" t="n"/>
       <c r="F28" s="525" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G28" s="526" t="inlineStr">
         <is>
@@ -26918,7 +26904,7 @@
       </c>
       <c r="E29" s="99" t="n"/>
       <c r="F29" s="525" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G29" s="526" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(kuru_tip): align Kuru Tip checklist items across templates, backend, CLI, Dart cell mappings, and mobile UI
</commit_message>
<xml_diff>
--- a/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
+++ b/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
@@ -2910,7 +2910,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3063,7 +3063,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -3108,7 +3108,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3348,7 +3348,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3501,7 +3501,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -3546,7 +3546,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3626,7 +3626,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3695,7 +3695,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3787,7 +3787,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3905,7 +3905,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3988,7 +3988,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4057,7 +4057,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4149,7 +4149,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4267,7 +4267,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4357,7 +4357,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4430,7 +4430,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4522,7 +4522,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4640,7 +4640,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4723,7 +4723,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4820,7 +4820,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t>None</a:t>
+                  <a:t/>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4932,7 +4932,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -4994,7 +4994,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -5033,7 +5033,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -6664,11 +6664,25 @@
     <row r="30" s="227"/>
     <row r="31"/>
     <row r="32" ht="11.25" customHeight="1" s="227"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40" s="227"/>
     <row r="41" s="227"/>
     <row r="42" s="227"/>
+    <row r="43"/>
     <row r="44" s="227"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
     <row r="48" ht="7.5" customHeight="1" s="227"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="481" t="n"/>
       <c r="B52" s="99" t="n"/>

</xml_diff>

<commit_message>
fix(templates): unmerge B43:S51 block on ANA SAYFA across all templates to prevent grounding values collision
</commit_message>
<xml_diff>
--- a/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
+++ b/backend/templates/HERMETİK TRAFO BAKIM RAPORU HİLMİ.xlsx
@@ -2910,7 +2910,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3063,7 +3063,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -3108,7 +3108,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3348,7 +3348,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3501,7 +3501,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -3546,7 +3546,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3626,7 +3626,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3695,7 +3695,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3787,7 +3787,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -3905,7 +3905,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -3988,7 +3988,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4057,7 +4057,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4149,7 +4149,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4267,7 +4267,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4357,7 +4357,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4430,7 +4430,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4522,7 +4522,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4640,7 +4640,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4723,7 +4723,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -4820,7 +4820,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="tr-TR"/>
               </a:p>
@@ -4932,7 +4932,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -4994,7 +4994,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="tr-TR"/>
           </a:p>
@@ -5033,7 +5033,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="tr-TR"/>
         </a:p>
@@ -6664,25 +6664,11 @@
     <row r="30" s="227"/>
     <row r="31"/>
     <row r="32" ht="11.25" customHeight="1" s="227"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40" s="227"/>
     <row r="41" s="227"/>
     <row r="42" s="227"/>
-    <row r="43"/>
     <row r="44" s="227"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
     <row r="48" ht="7.5" customHeight="1" s="227"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="481" t="n"/>
       <c r="B52" s="99" t="n"/>
@@ -18496,29 +18482,10 @@
     <row r="43" ht="3" customHeight="1" s="227">
       <c r="A43" s="10" t="n"/>
       <c r="B43" s="485" t="n"/>
-      <c r="C43" s="47" t="n"/>
-      <c r="D43" s="47" t="n"/>
-      <c r="E43" s="47" t="n"/>
-      <c r="F43" s="47" t="n"/>
-      <c r="G43" s="47" t="n"/>
-      <c r="H43" s="47" t="n"/>
-      <c r="I43" s="47" t="n"/>
-      <c r="J43" s="47" t="n"/>
-      <c r="K43" s="47" t="n"/>
-      <c r="L43" s="47" t="n"/>
-      <c r="M43" s="47" t="n"/>
-      <c r="N43" s="47" t="n"/>
-      <c r="O43" s="47" t="n"/>
-      <c r="P43" s="47" t="n"/>
-      <c r="Q43" s="47" t="n"/>
-      <c r="R43" s="47" t="n"/>
-      <c r="S43" s="211" t="n"/>
       <c r="T43" s="11" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="227">
       <c r="A44" s="10" t="n"/>
-      <c r="B44" s="62" t="n"/>
-      <c r="S44" s="212" t="n"/>
       <c r="T44" s="11" t="n"/>
       <c r="V44" s="485" t="inlineStr">
         <is>
@@ -18549,8 +18516,6 @@
     </row>
     <row r="45" ht="3" customHeight="1" s="227">
       <c r="A45" s="10" t="n"/>
-      <c r="B45" s="62" t="n"/>
-      <c r="S45" s="212" t="n"/>
       <c r="T45" s="11" t="n"/>
       <c r="V45" s="3" t="n"/>
       <c r="W45" s="127" t="n"/>
@@ -18573,8 +18538,6 @@
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
-      <c r="B46" s="62" t="n"/>
-      <c r="S46" s="212" t="n"/>
       <c r="T46" s="11" t="n"/>
       <c r="V46" s="489" t="inlineStr">
         <is>
@@ -18621,8 +18584,6 @@
     </row>
     <row r="47" ht="3" customHeight="1" s="227">
       <c r="A47" s="10" t="n"/>
-      <c r="B47" s="62" t="n"/>
-      <c r="S47" s="212" t="n"/>
       <c r="T47" s="11" t="n"/>
       <c r="V47" s="3" t="n"/>
       <c r="W47" s="127" t="n"/>
@@ -18645,8 +18606,6 @@
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
-      <c r="B48" s="62" t="n"/>
-      <c r="S48" s="212" t="n"/>
       <c r="T48" s="11" t="n"/>
       <c r="V48" s="490">
         <f>V57/1.0525889</f>
@@ -18687,8 +18646,6 @@
     </row>
     <row r="49" ht="3" customHeight="1" s="227">
       <c r="A49" s="10" t="n"/>
-      <c r="B49" s="62" t="n"/>
-      <c r="S49" s="212" t="n"/>
       <c r="T49" s="11" t="n"/>
       <c r="V49" s="42" t="n"/>
       <c r="W49" s="43" t="n"/>
@@ -18711,8 +18668,6 @@
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
-      <c r="B50" s="62" t="n"/>
-      <c r="S50" s="212" t="n"/>
       <c r="T50" s="11" t="n"/>
       <c r="V50" s="328" t="inlineStr">
         <is>
@@ -18759,24 +18714,6 @@
     </row>
     <row r="51" ht="3" customHeight="1" s="227">
       <c r="A51" s="10" t="n"/>
-      <c r="B51" s="49" t="n"/>
-      <c r="C51" s="50" t="n"/>
-      <c r="D51" s="50" t="n"/>
-      <c r="E51" s="50" t="n"/>
-      <c r="F51" s="50" t="n"/>
-      <c r="G51" s="50" t="n"/>
-      <c r="H51" s="50" t="n"/>
-      <c r="I51" s="50" t="n"/>
-      <c r="J51" s="50" t="n"/>
-      <c r="K51" s="50" t="n"/>
-      <c r="L51" s="50" t="n"/>
-      <c r="M51" s="50" t="n"/>
-      <c r="N51" s="50" t="n"/>
-      <c r="O51" s="50" t="n"/>
-      <c r="P51" s="50" t="n"/>
-      <c r="Q51" s="50" t="n"/>
-      <c r="R51" s="50" t="n"/>
-      <c r="S51" s="213" t="n"/>
       <c r="T51" s="11" t="n"/>
     </row>
     <row r="52" ht="3" customHeight="1" s="227">
@@ -20011,7 +19948,7 @@
       <c r="T83" s="17" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="161">
+  <mergeCells count="160">
     <mergeCell ref="G55:J55"/>
     <mergeCell ref="F68:G68"/>
     <mergeCell ref="AL57:AN57"/>
@@ -20023,7 +19960,6 @@
     <mergeCell ref="L68:M68"/>
     <mergeCell ref="K5:S6"/>
     <mergeCell ref="V66:X66"/>
-    <mergeCell ref="B43:S51"/>
     <mergeCell ref="K17:M17"/>
     <mergeCell ref="I66:J66"/>
     <mergeCell ref="K33:N33"/>

</xml_diff>